<commit_message>
Milestone 3C Saudi QR and visual PDF
</commit_message>
<xml_diff>
--- a/test_data/workbooks/SA-VALID-001.xlsx
+++ b/test_data/workbooks/SA-VALID-001.xlsx
@@ -527,7 +527,6 @@
           <t>billing@example.test</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -890,7 +889,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L2"/>
+  <dimension ref="A1:M2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -911,45 +910,50 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
+          <t>description_ar</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
           <t>item_name</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>quantity</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>unit_code</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>unit_price</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>line_net_amount</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>tax_category_code</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>tax_rate</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>tax_amount</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>line_gross_amount</t>
         </is>
@@ -971,35 +975,40 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
+          <t>خدمات استشارية</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
           <t>Consulting services</t>
         </is>
       </c>
-      <c r="E2" t="n">
+      <c r="F2" t="n">
         <v>10</v>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>HUR</t>
         </is>
       </c>
-      <c r="G2" t="n">
+      <c r="H2" t="n">
         <v>1000</v>
       </c>
-      <c r="H2" t="n">
+      <c r="I2" t="n">
         <v>10000</v>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t>S</t>
         </is>
       </c>
-      <c r="J2" t="n">
+      <c r="K2" t="n">
         <v>15</v>
       </c>
-      <c r="K2" t="n">
+      <c r="L2" t="n">
         <v>1500</v>
       </c>
-      <c r="L2" t="n">
+      <c r="M2" t="n">
         <v>11500</v>
       </c>
     </row>

</xml_diff>